<commit_message>
Planning out 75mm guns
</commit_message>
<xml_diff>
--- a/toi/documentation/Demarre Penetration Calculator.xlsx
+++ b/toi/documentation/Demarre Penetration Calculator.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\EoaNBR\EoaNBR\toi\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\EoaNBR\EoaNBR\toi\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Reference pen</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Pen Constant in mm</t>
+  </si>
+  <si>
+    <t>47mm basis</t>
+  </si>
+  <si>
+    <t>57mm basis</t>
   </si>
 </sst>
 </file>
@@ -377,69 +383,100 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:B16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.140625" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
         <v>46.122999999999998</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <f>(B11)</f>
+        <v>52.31226744964134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
         <v>574</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7">
         <v>538</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
         <v>57</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9">
         <v>2.72</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>5.87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -447,8 +484,12 @@
         <f>(B2*((B7/B3)^1.4283)*((B8/B4)^1.0714)*(((B9/(B8^3))^0.7143)/((B5/(B4^3))^0.7143)))</f>
         <v>52.31226744964134</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <f>(C2*((C7/C3)^1.4283)*((C8/C4)^1.0714)*(((C9/(C8^3))^0.7143)/((C5/(C4^3))^0.7143)))</f>
+        <v>94.564609179276715</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -456,8 +497,12 @@
         <f>(B11/25.4)</f>
         <v>2.0595380885685568</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <f>(C11/25.4)</f>
+        <v>3.7230161094203433</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -465,8 +510,12 @@
         <f>(7.7/14.12)</f>
         <v>0.54532577903682722</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <f>(7.7/14.12)</f>
+        <v>0.54532577903682722</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -474,14 +523,22 @@
         <f>(B14 * 25.4)</f>
         <v>13.851274787535411</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <f>(C14 * 25.4)</f>
+        <v>13.851274787535411</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>
       <c r="B16">
         <f>(B11 / B15)</f>
         <v>3.7767114039724698</v>
+      </c>
+      <c r="C16">
+        <f>(C11 / C15)</f>
+        <v>6.8271412292227591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>